<commit_message>
Update demos to the latest version 26.1
</commit_message>
<xml_diff>
--- a/Data/LoanCalculator.xlsx
+++ b/Data/LoanCalculator.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DX\2016.2\Demos.RealLife\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bugs\FromTesting\Demo-Products\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC33C371-34E4-47BF-A95E-3E5206EA905A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="105" windowWidth="27795" windowHeight="12600"/>
+    <workbookView xWindow="31040" yWindow="-8590" windowWidth="25530" windowHeight="16170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Loan Calculator" sheetId="1" r:id="rId1"/>
@@ -40,7 +41,20 @@
     <definedName name="TradeIn">'Loan Calculator'!$D$6</definedName>
     <definedName name="TradeInOwed">'Loan Calculator'!$D$7</definedName>
   </definedNames>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -146,7 +160,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="6">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -167,20 +181,20 @@
       <sz val="36"/>
       <color theme="3"/>
       <name val="Arial Black"/>
-      <charset val="204"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="16"/>
       <color theme="0"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="16"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -188,21 +202,21 @@
       <sz val="11"/>
       <color theme="3"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="16"/>
       <color theme="5"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="16"/>
       <color theme="6"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -210,7 +224,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -218,13 +232,14 @@
       <sz val="18"/>
       <color theme="3"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="16"/>
       <color theme="4"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -232,7 +247,7 @@
       <sz val="10"/>
       <color theme="3"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -240,7 +255,7 @@
       <sz val="28"/>
       <color theme="5"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -248,7 +263,7 @@
       <sz val="9"/>
       <color theme="3"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -256,7 +271,7 @@
       <sz val="10"/>
       <color theme="3"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -264,7 +279,7 @@
       <sz val="28"/>
       <color theme="6"/>
       <name val="Century Gothic"/>
-      <charset val="204"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -272,12 +287,14 @@
       <sz val="13"/>
       <color theme="3"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -285,6 +302,7 @@
       <sz val="15"/>
       <color theme="3"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -326,7 +344,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -573,6 +591,67 @@
       <top/>
       <bottom style="thick">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="dashed">
+        <color theme="0" tint="-0.24994659260841701"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thick">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -593,7 +672,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1">
@@ -611,36 +690,28 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="8" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="8" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="8" fontId="4" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -665,13 +736,10 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="8" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
@@ -698,7 +766,7 @@
     <xf numFmtId="8" fontId="4" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -710,16 +778,16 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="14" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -728,7 +796,7 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="8" fontId="4" fillId="5" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -737,13 +805,12 @@
     <xf numFmtId="8" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="10" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -752,11 +819,10 @@
     <xf numFmtId="8" fontId="7" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="8" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="8" fontId="10" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -768,15 +834,40 @@
     <xf numFmtId="8" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="8" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="8" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="4" fillId="5" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
     <xf numFmtId="166" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
@@ -793,6 +884,35 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -805,7 +925,7 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -814,12 +934,6 @@
     <xf numFmtId="167" fontId="11" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
@@ -832,30 +946,14 @@
     <xf numFmtId="167" fontId="14" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="8">
-    <cellStyle name="Auto Loan Info Header" xfId="2"/>
+    <cellStyle name="Auto Loan Info Header" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Comma" xfId="5" builtinId="3"/>
-    <cellStyle name="General Loan Info Header" xfId="1"/>
+    <cellStyle name="General Loan Info Header" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Heading 1" xfId="7" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="4" builtinId="17"/>
-    <cellStyle name="Home Equity Info Header" xfId="3"/>
+    <cellStyle name="Home Equity Info Header" xfId="3" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
     <cellStyle name="Title" xfId="6" builtinId="15"/>
   </cellStyles>
@@ -1102,465 +1200,468 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:O28"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1.5" customWidth="1"/>
     <col min="2" max="2" width="2.5" customWidth="1"/>
     <col min="3" max="3" width="34.5" customWidth="1"/>
-    <col min="4" max="4" width="12.375" customWidth="1"/>
-    <col min="5" max="5" width="2.375" customWidth="1"/>
+    <col min="4" max="4" width="12.3984375" customWidth="1"/>
+    <col min="5" max="5" width="2.3984375" customWidth="1"/>
     <col min="6" max="6" width="2" customWidth="1"/>
     <col min="7" max="7" width="2.5" customWidth="1"/>
-    <col min="8" max="8" width="27.375" customWidth="1"/>
-    <col min="9" max="9" width="12.375" customWidth="1"/>
-    <col min="10" max="10" width="2.25" customWidth="1"/>
+    <col min="8" max="8" width="27.3984375" customWidth="1"/>
+    <col min="9" max="9" width="12.3984375" customWidth="1"/>
+    <col min="10" max="10" width="2.19921875" customWidth="1"/>
     <col min="11" max="11" width="2" customWidth="1"/>
     <col min="12" max="12" width="2.5" customWidth="1"/>
-    <col min="13" max="13" width="32.25" customWidth="1"/>
-    <col min="14" max="14" width="12.375" customWidth="1"/>
-    <col min="15" max="15" width="2.25" customWidth="1"/>
+    <col min="13" max="13" width="32.19921875" customWidth="1"/>
+    <col min="14" max="14" width="12.3984375" customWidth="1"/>
+    <col min="15" max="15" width="2.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:15" ht="55.5" x14ac:dyDescent="1.05">
+    <row r="1" spans="2:15" ht="55.2" x14ac:dyDescent="1.3">
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:15" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:15" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2"/>
-      <c r="C3" s="70" t="s">
+      <c r="C3" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="70"/>
+      <c r="D3" s="74"/>
       <c r="E3" s="2"/>
       <c r="G3" s="3"/>
-      <c r="H3" s="71" t="s">
+      <c r="H3" s="75" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="71"/>
+      <c r="I3" s="75"/>
       <c r="J3" s="4"/>
+      <c r="K3" s="69"/>
       <c r="L3" s="5"/>
-      <c r="M3" s="72" t="s">
+      <c r="M3" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="72"/>
+      <c r="N3" s="76"/>
       <c r="O3" s="5"/>
     </row>
-    <row r="4" spans="2:15" ht="19.5" x14ac:dyDescent="0.3">
-      <c r="B4" s="6"/>
-      <c r="C4" s="7" t="s">
+    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.25">
+      <c r="B4" s="62"/>
+      <c r="C4" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="64">
         <v>45000</v>
       </c>
-      <c r="E4" s="9"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="87" t="s">
+      <c r="E4" s="65"/>
+      <c r="G4" s="70"/>
+      <c r="H4" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="88">
+      <c r="I4" s="80">
         <v>5.5E-2</v>
       </c>
-      <c r="J4" s="13"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="7" t="s">
+      <c r="J4" s="71"/>
+      <c r="K4" s="72"/>
+      <c r="L4" s="66"/>
+      <c r="M4" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="15">
+      <c r="N4" s="67">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="O4" s="16"/>
-    </row>
-    <row r="5" spans="2:15" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O4" s="68"/>
+    </row>
+    <row r="5" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="6"/>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="16">
         <v>2000</v>
       </c>
-      <c r="E5" s="9"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="87"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="13"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="17" t="s">
+      <c r="E5" s="8"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="79"/>
+      <c r="I5" s="81"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="72"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="N5" s="18">
+      <c r="N5" s="16">
         <v>2000</v>
       </c>
-      <c r="O5" s="16"/>
-    </row>
-    <row r="6" spans="2:15" ht="20.25" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="O5" s="14"/>
+    </row>
+    <row r="6" spans="2:15" ht="21.6" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B6" s="6"/>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="16">
         <v>15000</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="89" t="s">
+      <c r="E6" s="8"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="85" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="89"/>
-      <c r="J6" s="20"/>
-      <c r="L6" s="14"/>
-      <c r="M6" s="17" t="s">
+      <c r="I6" s="85"/>
+      <c r="J6" s="18"/>
+      <c r="L6" s="13"/>
+      <c r="M6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="N6" s="21">
+      <c r="N6" s="19">
         <v>0.17</v>
       </c>
-      <c r="O6" s="16"/>
-    </row>
-    <row r="7" spans="2:15" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O6" s="14"/>
+    </row>
+    <row r="7" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6"/>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="16">
         <v>13000</v>
       </c>
-      <c r="E7" s="9"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="90"/>
-      <c r="I7" s="90"/>
-      <c r="J7" s="23"/>
-      <c r="L7" s="14"/>
-      <c r="M7" s="11" t="s">
+      <c r="E7" s="8"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="86"/>
+      <c r="I7" s="86"/>
+      <c r="J7" s="21"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="N7" s="12">
+      <c r="N7" s="11">
         <v>0.09</v>
       </c>
-      <c r="O7" s="16"/>
-    </row>
-    <row r="8" spans="2:15" ht="20.25" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="O7" s="14"/>
+    </row>
+    <row r="8" spans="2:15" ht="21.6" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B8" s="6"/>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="22">
         <v>60</v>
       </c>
-      <c r="E8" s="25"/>
-      <c r="G8" s="14"/>
+      <c r="E8" s="23"/>
+      <c r="G8" s="13"/>
       <c r="H8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="26">
+      <c r="I8" s="24">
         <f>IFERROR(ROUND(PMT(LoanInterestRate/12,Term,-AutoLoanAmount),2),"")</f>
         <v>833.86</v>
       </c>
-      <c r="J8" s="27"/>
-      <c r="L8" s="28"/>
-      <c r="M8" s="81" t="s">
+      <c r="J8" s="8"/>
+      <c r="L8" s="25"/>
+      <c r="M8" s="83" t="s">
         <v>16</v>
       </c>
-      <c r="N8" s="81"/>
-      <c r="O8" s="29"/>
-    </row>
-    <row r="9" spans="2:15" ht="19.5" x14ac:dyDescent="0.3">
+      <c r="N8" s="83"/>
+      <c r="O8" s="26"/>
+    </row>
+    <row r="9" spans="2:15" ht="21" x14ac:dyDescent="0.25">
       <c r="B9" s="6"/>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="19">
         <v>8.7499999999999994E-2</v>
       </c>
-      <c r="E9" s="13"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="17" t="str">
+      <c r="E9" s="12"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="15" t="str">
         <f>"Total interest ("&amp;TEXT(LoanInterestRate,"0.00%")&amp;")"</f>
         <v>Total interest (5.50%)</v>
       </c>
-      <c r="I9" s="31">
+      <c r="I9" s="28">
         <f>IFERROR((AutoMonthlyPayment*Term)-AutoLoanAmount,"")</f>
         <v>6376.5999999999985</v>
       </c>
-      <c r="J9" s="32"/>
-      <c r="L9" s="33"/>
-      <c r="M9" s="82"/>
-      <c r="N9" s="82"/>
-      <c r="O9" s="34"/>
-    </row>
-    <row r="10" spans="2:15" ht="19.5" x14ac:dyDescent="0.3">
+      <c r="J9" s="29"/>
+      <c r="L9" s="30"/>
+      <c r="M9" s="84"/>
+      <c r="N9" s="84"/>
+      <c r="O9" s="31"/>
+    </row>
+    <row r="10" spans="2:15" ht="21" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="16">
         <v>30</v>
       </c>
-      <c r="E10" s="9"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="17" t="s">
+      <c r="E10" s="8"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="35">
+      <c r="I10" s="32">
         <v>0</v>
       </c>
-      <c r="J10" s="27"/>
-      <c r="L10" s="14"/>
+      <c r="J10" s="8"/>
+      <c r="L10" s="13"/>
       <c r="M10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N10" s="26">
+      <c r="N10" s="24">
         <f>IFERROR(ROUND(PMT(EquityInterestRate/12,Term,-EquityLoanAmount),2),"")</f>
         <v>851.15</v>
       </c>
-      <c r="O10" s="16"/>
-    </row>
-    <row r="11" spans="2:15" ht="19.5" x14ac:dyDescent="0.3">
+      <c r="O10" s="14"/>
+    </row>
+    <row r="11" spans="2:15" ht="21" x14ac:dyDescent="0.25">
       <c r="B11" s="6"/>
-      <c r="C11" s="91" t="s">
+      <c r="C11" s="82" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="69" t="s">
+      <c r="D11" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="36"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="17" t="s">
+      <c r="E11" s="33"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="I11" s="35">
+      <c r="I11" s="32">
         <f>IFERROR((AutoMonthlyPayment*Term),"")</f>
         <v>50031.6</v>
       </c>
-      <c r="J11" s="27"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="17" t="str">
+      <c r="J11" s="8"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="15" t="str">
         <f>"Total Loan interest ("&amp;TEXT(EquityInterestRate,"0.00%")&amp;")"</f>
         <v>Total Loan interest (4.50%)</v>
       </c>
-      <c r="N11" s="31">
+      <c r="N11" s="28">
         <f>IFERROR((EquityMonthlyPayment*Term)-EquityLoanAmount,"")</f>
         <v>5414</v>
       </c>
-      <c r="O11" s="16"/>
-    </row>
-    <row r="12" spans="2:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="37"/>
-      <c r="C12" s="91"/>
-      <c r="D12" s="69"/>
-      <c r="E12" s="36"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="11" t="s">
+      <c r="O11" s="14"/>
+    </row>
+    <row r="12" spans="2:15" ht="24" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="34"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="73"/>
+      <c r="E12" s="33"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="I12" s="38">
+      <c r="I12" s="35">
         <f>AutoTotalInterest</f>
         <v>6376.5999999999985</v>
       </c>
-      <c r="J12" s="16"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="17" t="s">
+      <c r="J12" s="14"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="N12" s="35">
+      <c r="N12" s="32">
         <f>IFERROR(EquityTotalInterest*(FederalTaxRate+StateTaxRate),"")</f>
         <v>1407.64</v>
       </c>
-      <c r="O12" s="16"/>
-    </row>
-    <row r="13" spans="2:15" ht="23.25" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="39"/>
-      <c r="C13" s="75" t="s">
+      <c r="O12" s="14"/>
+    </row>
+    <row r="13" spans="2:15" ht="24" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="36"/>
+      <c r="C13" s="88" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="75"/>
-      <c r="E13" s="40"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="77" t="s">
+      <c r="D13" s="88"/>
+      <c r="E13" s="37"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="90" t="s">
         <v>25</v>
       </c>
-      <c r="I13" s="77"/>
-      <c r="J13" s="41"/>
-      <c r="L13" s="14"/>
-      <c r="M13" s="17" t="s">
+      <c r="I13" s="90"/>
+      <c r="J13" s="38"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="N13" s="35">
+      <c r="N13" s="32">
         <f>IFERROR((EquityMonthlyPayment*Term),"")</f>
         <v>51069</v>
       </c>
-      <c r="O13" s="16"/>
-    </row>
-    <row r="14" spans="2:15" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="42"/>
-      <c r="C14" s="76"/>
-      <c r="D14" s="76"/>
-      <c r="E14" s="43"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="78"/>
-      <c r="I14" s="78"/>
-      <c r="J14" s="45"/>
-      <c r="L14" s="14"/>
-      <c r="M14" s="46" t="s">
+      <c r="O13" s="14"/>
+    </row>
+    <row r="14" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="39"/>
+      <c r="C14" s="89"/>
+      <c r="D14" s="89"/>
+      <c r="E14" s="40"/>
+      <c r="G14" s="41"/>
+      <c r="H14" s="91"/>
+      <c r="I14" s="91"/>
+      <c r="J14" s="42"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="N14" s="47">
+      <c r="N14" s="44">
         <f>IFERROR(EquityTotalInterest-IncomeTaxSavings,"")</f>
         <v>4006.3599999999997</v>
       </c>
-      <c r="O14" s="16"/>
-    </row>
-    <row r="15" spans="2:15" ht="20.25" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="14"/>
+      <c r="O14" s="14"/>
+    </row>
+    <row r="15" spans="2:15" ht="21.6" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="13"/>
       <c r="C15" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="48">
+      <c r="D15" s="45">
         <f>PurchasePrice</f>
         <v>45000</v>
       </c>
-      <c r="E15" s="27"/>
-      <c r="G15" s="49"/>
-      <c r="H15" s="79">
+      <c r="E15" s="8"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="92">
         <f>AutoCostofLoan</f>
         <v>6376.5999999999985</v>
       </c>
-      <c r="I15" s="50"/>
-      <c r="J15" s="16"/>
-      <c r="L15" s="51"/>
-      <c r="M15" s="81" t="s">
+      <c r="I15" s="46"/>
+      <c r="J15" s="14"/>
+      <c r="L15" s="47"/>
+      <c r="M15" s="83" t="s">
         <v>25</v>
       </c>
-      <c r="N15" s="81"/>
-      <c r="O15" s="29"/>
-    </row>
-    <row r="16" spans="2:15" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="14"/>
-      <c r="C16" s="17" t="s">
+      <c r="N15" s="83"/>
+      <c r="O15" s="26"/>
+    </row>
+    <row r="16" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="13"/>
+      <c r="C16" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="52">
+      <c r="D16" s="48">
         <f>IF(SalesTaxDeduciton="Yes",(PurchasePrice-TradeIn)*SalesTaxRate,AutoPurchaseAmount*SalesTaxRate)</f>
         <v>2625</v>
       </c>
-      <c r="E16" s="27"/>
-      <c r="G16" s="53"/>
-      <c r="H16" s="80"/>
-      <c r="I16" s="54"/>
-      <c r="J16" s="55"/>
-      <c r="L16" s="33"/>
-      <c r="M16" s="82"/>
-      <c r="N16" s="82"/>
-      <c r="O16" s="34"/>
-    </row>
-    <row r="17" spans="2:15" ht="17.25" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="14"/>
-      <c r="C17" s="83" t="str">
+      <c r="E16" s="8"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="93"/>
+      <c r="I16" s="50"/>
+      <c r="J16" s="51"/>
+      <c r="L16" s="30"/>
+      <c r="M16" s="84"/>
+      <c r="N16" s="84"/>
+      <c r="O16" s="31"/>
+    </row>
+    <row r="17" spans="2:15" ht="14.4" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="13"/>
+      <c r="C17" s="94" t="str">
         <f>IF(AND(SalesTaxDeduciton="Yes",SalesTaxAmount&gt;0),"Sales tax based on "&amp;TEXT((PurchasePrice-TradeIn),"$#,##0.00")&amp;" (sales tax deduction for trade-in allowance)","")</f>
         <v>Sales tax based on $30,000.00 (sales tax deduction for trade-in allowance)</v>
       </c>
-      <c r="D17" s="56"/>
-      <c r="E17" s="57"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="85">
+      <c r="D17" s="52"/>
+      <c r="E17" s="53"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="96">
         <f>EquityCostofLoan</f>
         <v>4006.3599999999997</v>
       </c>
-      <c r="N17" s="50"/>
-      <c r="O17" s="16"/>
-    </row>
-    <row r="18" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="14"/>
-      <c r="C18" s="84"/>
-      <c r="D18" s="58"/>
-      <c r="E18" s="27"/>
-      <c r="L18" s="59"/>
-      <c r="M18" s="86"/>
-      <c r="N18" s="54"/>
-      <c r="O18" s="55"/>
-    </row>
-    <row r="19" spans="2:15" ht="17.25" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="14"/>
-      <c r="C19" s="17" t="s">
+      <c r="N17" s="46"/>
+      <c r="O17" s="14"/>
+    </row>
+    <row r="18" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="13"/>
+      <c r="C18" s="95"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="8"/>
+      <c r="L18" s="49"/>
+      <c r="M18" s="97"/>
+      <c r="N18" s="50"/>
+      <c r="O18" s="51"/>
+    </row>
+    <row r="19" spans="2:15" ht="14.4" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="13"/>
+      <c r="C19" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="D19" s="52">
+      <c r="D19" s="48">
         <f>CashDown+(TradeIn-TradeInOwed)</f>
         <v>4000</v>
       </c>
-      <c r="E19" s="27"/>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B20" s="14"/>
-      <c r="C20" s="73" t="str">
+      <c r="E19" s="8"/>
+    </row>
+    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B20" s="13"/>
+      <c r="C20" s="77" t="str">
         <f>IF(TradeIn&gt;0,"Total down payment calculation includes "&amp;IF(TradeInOwed&gt;0,TEXT(TradeIn-TradeInOwed,"$#,##0.00")&amp;" ("&amp;TEXT(TradeIn,"$#,##0.00")&amp;" trade-in amount minus "&amp;TEXT(TradeInOwed,"$#,##0.00")&amp;" outstanding loan balance)",TEXT(TradeIn,"$#,##0.00")&amp;" trade-in amount")&amp;IF(CashDown&gt;0," plus "&amp;TEXT(CashDown,"$#,##0.00")&amp;" cash down",""),IF(CashDown&gt;0,"Down payment calculation includes " &amp; TEXT(CashDown,"$#,##0.00") &amp; " cash down",""))</f>
         <v>Total down payment calculation includes $2,000.00 ($15,000.00 trade-in amount minus $13,000.00 outstanding loan balance) plus $2,000.00 cash down</v>
       </c>
-      <c r="D20" s="73"/>
-      <c r="E20" s="27"/>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B21" s="14"/>
-      <c r="C21" s="73"/>
-      <c r="D21" s="73"/>
-      <c r="E21" s="27"/>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B22" s="14"/>
-      <c r="C22" s="73"/>
-      <c r="D22" s="73"/>
-      <c r="E22" s="27"/>
-    </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B23" s="14"/>
-      <c r="C23" s="60" t="s">
+      <c r="D20" s="77"/>
+      <c r="E20" s="8"/>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B21" s="13"/>
+      <c r="C21" s="77"/>
+      <c r="D21" s="77"/>
+      <c r="E21" s="8"/>
+    </row>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B22" s="13"/>
+      <c r="C22" s="77"/>
+      <c r="D22" s="77"/>
+      <c r="E22" s="8"/>
+    </row>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B23" s="13"/>
+      <c r="C23" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="D23" s="61">
+      <c r="D23" s="56">
         <f>(AutoPurchaseAmount+SalesTaxAmount+LoanFees)-CashDown-(TradeIn-TradeInOwed)</f>
         <v>43655</v>
       </c>
-      <c r="E23" s="27"/>
-    </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B24" s="14"/>
-      <c r="C24" s="62" t="str">
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B24" s="13"/>
+      <c r="C24" s="57" t="str">
         <f>IF(LoanFees&gt;0,"Includes " &amp;TEXT(LoanFees,"$#,##0.00") &amp; " for fees","")</f>
         <v>Includes $30.00 for fees</v>
       </c>
-      <c r="D24" s="63"/>
-      <c r="E24" s="27"/>
-    </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B25" s="14"/>
-      <c r="C25" s="64" t="s">
+      <c r="D24" s="58"/>
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B25" s="13"/>
+      <c r="C25" s="59" t="s">
         <v>31</v>
       </c>
-      <c r="D25" s="65">
+      <c r="D25" s="60">
         <f>(AutoPurchaseAmount+SalesTaxAmount+LoanFees+ClosingCosts)-CashDown-(TradeIn-TradeInOwed)</f>
         <v>45655</v>
       </c>
-      <c r="E25" s="27"/>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B26" s="14"/>
-      <c r="C26" s="73" t="str">
+      <c r="E25" s="8"/>
+    </row>
+    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B26" s="13"/>
+      <c r="C26" s="77" t="str">
         <f>IF(ClosingCosts&gt;0,"Includes " &amp;TEXT(LoanFees+ClosingCosts,"$#,##0.00") &amp; " for fees and closing costs","")</f>
         <v>Includes $2,030.00 for fees and closing costs</v>
       </c>
-      <c r="D26" s="66"/>
-      <c r="E26" s="67"/>
-    </row>
-    <row r="27" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="59"/>
-      <c r="C27" s="74"/>
-      <c r="D27" s="68"/>
-      <c r="E27" s="55"/>
-    </row>
-    <row r="28" spans="2:15" ht="17.25" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="61"/>
+    </row>
+    <row r="27" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="49"/>
+      <c r="C27" s="87"/>
+      <c r="D27" s="50"/>
+      <c r="E27" s="51"/>
+    </row>
+    <row r="28" spans="2:15" ht="14.4" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="C26:C27"/>
@@ -1591,7 +1692,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please select Yes or No from the list." sqref="D11:E11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please select Yes or No from the list." sqref="D11:E11" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>